<commit_message>
Rename notebook HDBSCAN, tambah dataset_kontrol, update output perbandingan
</commit_message>
<xml_diff>
--- a/uts/outputPerbandingan/perbandingan_3_algoritma.xlsx
+++ b/uts/outputPerbandingan/perbandingan_3_algoritma.xlsx
@@ -772,7 +772,7 @@
         <v>1312.88</v>
       </c>
       <c r="K8" t="n">
-        <v>154.28839</v>
+        <v>141.28673</v>
       </c>
     </row>
     <row r="9">
@@ -813,7 +813,7 @@
         <v>1444.43</v>
       </c>
       <c r="K9" t="n">
-        <v>139.96335</v>
+        <v>74.60652</v>
       </c>
     </row>
     <row r="10">
@@ -854,7 +854,7 @@
         <v>1890.15</v>
       </c>
       <c r="K10" t="n">
-        <v>118.49736</v>
+        <v>62.12746</v>
       </c>
     </row>
   </sheetData>
@@ -1014,7 +1014,7 @@
         <v>1312.88</v>
       </c>
       <c r="I4" t="n">
-        <v>154.28839</v>
+        <v>141.28673</v>
       </c>
     </row>
   </sheetData>
@@ -1174,7 +1174,7 @@
         <v>1444.43</v>
       </c>
       <c r="I4" t="n">
-        <v>139.96335</v>
+        <v>74.60652</v>
       </c>
     </row>
   </sheetData>
@@ -1334,7 +1334,7 @@
         <v>1890.15</v>
       </c>
       <c r="I4" t="n">
-        <v>118.49736</v>
+        <v>62.12746</v>
       </c>
     </row>
   </sheetData>

</xml_diff>